<commit_message>
Remove placeholder subjects; keep Status/Priority dropdowns
Clears the sample subject rows (Mathematics/Physics/Chemistry/Biology)
from the Tracker and Dashboard so the template starts blank. Status,
Priority, and Confidence remain dropdown-driven via the Lists sheet.

https://claude.ai/code/session_01D6ynHXdt2652kY5oWwKy8A
</commit_message>
<xml_diff>
--- a/Study_Progress_Tracker.xlsx
+++ b/Study_Progress_Tracker.xlsx
@@ -852,11 +852,7 @@
       <c r="F12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
+      <c r="B13" s="14" t="inlineStr"/>
       <c r="C13" s="15">
         <f>IF($B13="","",COUNTIF(Tracker!$A$4:$A$203,$B13))</f>
         <v/>
@@ -872,11 +868,7 @@
       <c r="F13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Physics</t>
-        </is>
-      </c>
+      <c r="B14" s="14" t="inlineStr"/>
       <c r="C14" s="15">
         <f>IF($B14="","",COUNTIF(Tracker!$A$4:$A$203,$B14))</f>
         <v/>
@@ -892,11 +884,7 @@
       <c r="F14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>Chemistry</t>
-        </is>
-      </c>
+      <c r="B15" s="14" t="inlineStr"/>
       <c r="C15" s="15">
         <f>IF($B15="","",COUNTIF(Tracker!$A$4:$A$203,$B15))</f>
         <v/>
@@ -912,11 +900,7 @@
       <c r="F15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
+      <c r="B16" s="14" t="inlineStr"/>
       <c r="C16" s="15">
         <f>IF($B16="","",COUNTIF(Tracker!$A$4:$A$203,$B16))</f>
         <v/>
@@ -1128,260 +1112,84 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="B4" s="21" t="inlineStr">
-        <is>
-          <t>Algebra - Quadratic Equations</t>
-        </is>
-      </c>
-      <c r="C4" s="22" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D4" s="22" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="E4" s="23" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="F4" s="23" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="G4" s="24" t="n">
-        <v>6</v>
-      </c>
-      <c r="H4" s="24" t="n">
-        <v>6</v>
-      </c>
+      <c r="A4" s="21" t="n"/>
+      <c r="B4" s="21" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="23" t="n"/>
+      <c r="F4" s="23" t="n"/>
+      <c r="G4" s="24" t="n"/>
+      <c r="H4" s="24" t="n"/>
       <c r="I4" s="25">
         <f>IF($A4="","",IF(D4="Completed",1,IF(D4="Revising",0.9,IF(D4="In Progress",IF($G4&gt;0,MIN(1,$H4/$G4),0.5),IF(D4="On Hold",0.25,0)))))</f>
         <v/>
       </c>
-      <c r="J4" s="22" t="inlineStr">
-        <is>
-          <t>4 - Good</t>
-        </is>
-      </c>
-      <c r="K4" s="21" t="inlineStr">
-        <is>
-          <t>Felt solid on practice set.</t>
-        </is>
-      </c>
+      <c r="J4" s="22" t="n"/>
+      <c r="K4" s="21" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="B5" s="26" t="inlineStr">
-        <is>
-          <t>Calculus - Integration</t>
-        </is>
-      </c>
-      <c r="C5" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="E5" s="28" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="F5" s="28" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="G5" s="29" t="n">
-        <v>8</v>
-      </c>
-      <c r="H5" s="29" t="n">
-        <v>3</v>
-      </c>
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="26" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="28" t="n"/>
+      <c r="F5" s="28" t="n"/>
+      <c r="G5" s="29" t="n"/>
+      <c r="H5" s="29" t="n"/>
       <c r="I5" s="30">
         <f>IF($A5="","",IF(D5="Completed",1,IF(D5="Revising",0.9,IF(D5="In Progress",IF($G5&gt;0,MIN(1,$H5/$G5),0.5),IF(D5="On Hold",0.25,0)))))</f>
         <v/>
       </c>
-      <c r="J5" s="27" t="inlineStr">
-        <is>
-          <t>3 - OK</t>
-        </is>
-      </c>
-      <c r="K5" s="26" t="inlineStr">
-        <is>
-          <t>Revisit by-parts.</t>
-        </is>
-      </c>
+      <c r="J5" s="27" t="n"/>
+      <c r="K5" s="26" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>Physics</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Thermodynamics</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D6" s="22" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="G6" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="H6" s="24" t="n">
-        <v>0</v>
-      </c>
+      <c r="A6" s="21" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="23" t="n"/>
+      <c r="F6" s="23" t="n"/>
+      <c r="G6" s="24" t="n"/>
+      <c r="H6" s="24" t="n"/>
       <c r="I6" s="25">
         <f>IF($A6="","",IF(D6="Completed",1,IF(D6="Revising",0.9,IF(D6="In Progress",IF($G6&gt;0,MIN(1,$H6/$G6),0.5),IF(D6="On Hold",0.25,0)))))</f>
         <v/>
       </c>
-      <c r="J6" s="22" t="inlineStr">
-        <is>
-          <t>1 - Shaky</t>
-        </is>
-      </c>
-      <c r="K6" s="21" t="inlineStr"/>
+      <c r="J6" s="22" t="n"/>
+      <c r="K6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>Chemistry</t>
-        </is>
-      </c>
-      <c r="B7" s="26" t="inlineStr">
-        <is>
-          <t>Organic - Reaction Mechanisms</t>
-        </is>
-      </c>
-      <c r="C7" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D7" s="27" t="inlineStr">
-        <is>
-          <t>Revising</t>
-        </is>
-      </c>
-      <c r="E7" s="28" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="F7" s="28" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="G7" s="29" t="n">
-        <v>7</v>
-      </c>
-      <c r="H7" s="29" t="n">
-        <v>5</v>
-      </c>
+      <c r="A7" s="26" t="n"/>
+      <c r="B7" s="26" t="n"/>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="28" t="n"/>
+      <c r="F7" s="28" t="n"/>
+      <c r="G7" s="29" t="n"/>
+      <c r="H7" s="29" t="n"/>
       <c r="I7" s="30">
         <f>IF($A7="","",IF(D7="Completed",1,IF(D7="Revising",0.9,IF(D7="In Progress",IF($G7&gt;0,MIN(1,$H7/$G7),0.5),IF(D7="On Hold",0.25,0)))))</f>
         <v/>
       </c>
-      <c r="J7" s="27" t="inlineStr">
-        <is>
-          <t>3 - OK</t>
-        </is>
-      </c>
-      <c r="K7" s="26" t="inlineStr">
-        <is>
-          <t>Make flashcards.</t>
-        </is>
-      </c>
+      <c r="J7" s="27" t="n"/>
+      <c r="K7" s="26" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="B8" s="21" t="inlineStr">
-        <is>
-          <t>Genetics</t>
-        </is>
-      </c>
-      <c r="C8" s="22" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="D8" s="22" t="inlineStr">
-        <is>
-          <t>On Hold</t>
-        </is>
-      </c>
-      <c r="E8" s="23" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="F8" s="23" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="G8" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="H8" s="24" t="n">
-        <v>1</v>
-      </c>
+      <c r="A8" s="21" t="n"/>
+      <c r="B8" s="21" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="23" t="n"/>
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="24" t="n"/>
+      <c r="H8" s="24" t="n"/>
       <c r="I8" s="25">
         <f>IF($A8="","",IF(D8="Completed",1,IF(D8="Revising",0.9,IF(D8="In Progress",IF($G8&gt;0,MIN(1,$H8/$G8),0.5),IF(D8="On Hold",0.25,0)))))</f>
         <v/>
       </c>
-      <c r="J8" s="22" t="inlineStr">
-        <is>
-          <t>2 - Weak</t>
-        </is>
-      </c>
-      <c r="K8" s="21" t="inlineStr">
-        <is>
-          <t>After exams week.</t>
-        </is>
-      </c>
+      <c r="J8" s="22" t="n"/>
+      <c r="K8" s="21" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="26" t="n"/>

</xml_diff>